<commit_message>
Fix Total Inventory: replace Fossil SOH with Cambium SOH, rename Amazon Inventory to Cambium SO
</commit_message>
<xml_diff>
--- a/data/input/inventory_amazon_fossil.xlsx
+++ b/data/input/inventory_amazon_fossil.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 14\Fossil\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBB1351-B4C5-48DE-BF49-806A3D21C38A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -3298,6 +3298,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -3312,6 +3342,274 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3556,174 +3854,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3798,136 +3928,6 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -14887,142 +14887,140 @@
   <conditionalFormatting sqref="A234">
     <cfRule type="duplicateValues" dxfId="91" priority="228"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A234:A254">
+    <cfRule type="duplicateValues" dxfId="90" priority="844"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A252:A254">
-    <cfRule type="duplicateValues" dxfId="90" priority="229"/>
-    <cfRule type="duplicateValues" dxfId="89" priority="230"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="229"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="230"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A335:A341">
+    <cfRule type="duplicateValues" dxfId="87" priority="834"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="835"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="88" priority="821"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="821"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D123">
-    <cfRule type="duplicateValues" dxfId="87" priority="313"/>
-    <cfRule type="duplicateValues" dxfId="86" priority="314"/>
-    <cfRule type="duplicateValues" dxfId="85" priority="315" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="84" priority="316" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="83" priority="317" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="317" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="315" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="314"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="313"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="316" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D124:D127 D109:D122">
+    <cfRule type="duplicateValues" dxfId="79" priority="899"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="898" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="897"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="900" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D149">
-    <cfRule type="duplicateValues" dxfId="82" priority="308"/>
-    <cfRule type="duplicateValues" dxfId="81" priority="309"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="310" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="311" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="312" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="312" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="311" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="310" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="309"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="308"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D150:D152 D128:D148">
-    <cfRule type="duplicateValues" dxfId="77" priority="328"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="329" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="329" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="328"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D150:D152">
-    <cfRule type="duplicateValues" dxfId="75" priority="330"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="331" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="331" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="330"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D153:D161">
+    <cfRule type="duplicateValues" dxfId="66" priority="859"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="866" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="865" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="864"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="863"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="862"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="860"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="861"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D171:D196">
-    <cfRule type="duplicateValues" dxfId="73" priority="270"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="271"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="272" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="273" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="274" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="273" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="274" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="270"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="271"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="272" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D208:D221">
-    <cfRule type="duplicateValues" dxfId="68" priority="247"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="248"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="249" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="250" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="64" priority="251" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="251" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="250" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="247"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="248"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="249" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D222:D223">
-    <cfRule type="duplicateValues" dxfId="63" priority="285"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="286"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="287" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="288" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="289" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="289" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="288" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="287" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="286"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="285"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D224">
-    <cfRule type="duplicateValues" dxfId="58" priority="239"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="240"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="241"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="242"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="243"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="244"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="245" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="246" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="246" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="245" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="244"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="243"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="242"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="241"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="240"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="239"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D225:D231">
-    <cfRule type="duplicateValues" dxfId="50" priority="231"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="232"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="233"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="234"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="235"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="236"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="237" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="238" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="232"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="236"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="238" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="237" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="233"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="235"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="234"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="231"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D234:D239">
-    <cfRule type="duplicateValues" dxfId="42" priority="211"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="211"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D247:D251">
-    <cfRule type="duplicateValues" dxfId="41" priority="222"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="223"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="224" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="225" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="226" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="224" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="226" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="225" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="223"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="222"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D284">
-    <cfRule type="duplicateValues" dxfId="36" priority="110"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="111"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="112"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="113"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="114"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="115"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="116" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="117" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="110"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="117" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="116" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="114"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="113"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="112"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D342:D343">
+    <cfRule type="duplicateValues" dxfId="13" priority="836"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="837"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="839"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="840"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="841"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="842" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="843" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="838"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="28" priority="824"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="825" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="825" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="824"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="26" priority="819"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="820" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="820" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="819"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="24" priority="817"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="818" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A335:A341">
-    <cfRule type="duplicateValues" dxfId="22" priority="834"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A335:A341">
-    <cfRule type="duplicateValues" dxfId="21" priority="835"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D342:D343">
-    <cfRule type="duplicateValues" dxfId="20" priority="836"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="837"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="838"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="839"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="840"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="841"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="842" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="843" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A234:A254">
-    <cfRule type="duplicateValues" dxfId="12" priority="844"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D153:D161">
-    <cfRule type="duplicateValues" dxfId="11" priority="859"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="860"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="861"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="862"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="863"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="864"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="865" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="866" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D124:D127 D109:D122">
-    <cfRule type="duplicateValues" dxfId="3" priority="897"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="898" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="899"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="900" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="817"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="818" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>